<commit_message>
Consolidación final: ronda 2 del árbitro y del verificador aplicada; PDF del resumen regenerado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDwCFFTud391ebBMaJpdsw
</commit_message>
<xml_diff>
--- a/revision_externa/2_0/hoja_revision.xlsx
+++ b/revision_externa/2_0/hoja_revision.xlsx
@@ -1113,31 +1113,31 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>V17-AUD-DP-TIP-DELTA-TAE</t>
+          <t>V17-AUD-DP-TIP-CALIBRACION-SOLO-HIPOTECA</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Subida del tipo de las nuevas hipotecas (TAE), 2021T4 al máximo de 2023T3: 2,5 puntos porcentuales (2,3-2,5 puntos porcentuales) (2021T4-2023T3; data/processed/v8/nacional_q_v8.csv (tipo_hip_nuevas_tae, Banco de España); dato de 2023; C4)</t>
+          <t>Calibración: efecto del tipo hipotecario si solo se transmite a la parte de compras con hipoteca (52 %): -5,9 % del nivel de precios (-11,7 a -5,9 % del nivel de precios) (2022-2025; TIP-CALIBRACION-EFECTO-HIPOTECARIO × 52 % (BdE IA2025, p. 124); dato de 2025; C4)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2.5106</v>
+        <v>-5.9079</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2.2723</v>
+        <v>-11.7498</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2.5106</v>
+        <v>-5.9079</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>puntos porcentuales</t>
+          <t>% del nivel de precios</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2021T4-2023T3</t>
+          <t>2022-2025</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>data/processed/v8/nacional_q_v8.csv (tipo_hip_nuevas_tae, Banco de España)</t>
+          <t>TIP-CALIBRACION-EFECTO-HIPOTECARIO × 52 % (BdE IA2025, p. 124)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>BdE</t>
         </is>
       </c>
       <c r="K11" s="3">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>script de origen: output/v17/f5/hechos.json:V17-AUD-DP-TIP-DELTA-TAE</t>
+          <t>script de origen: output/v17/f5/hechos.json:V17-AUD-DP-TIP-CALIBRACION-SOLO-HIPOTECA</t>
         </is>
       </c>
       <c r="M11" s="4">
@@ -1175,31 +1175,27 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>V17-B5-PRECIO-RENTA</t>
+          <t>V17-DOC-OHB-GT-ALQUILER-BCN-2021</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Precio de la vivienda / renta bruta por hogar (años), último dato: 8,4 años (2026-06; Banco de España, Síntesis de indicadores del mercado de la vivienda (SI_1_5); dato de 2026-06; C4)</t>
+          <t>Viviendas de alquiler habitual de Barcelona ciudad en manos de grandes tenedores (104.958 de 290.416): 36,1 % del alquiler habitual de la ciudad (1-1-2021; Observatori Metropolità de l'Habitatge de Barcelona (O-HB); dato de 2021; C4)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>8.359999999999999</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>6.039</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>9.356999999999999</v>
-      </c>
+        <v>36.1</v>
+      </c>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>años</t>
+          <t>% del alquiler habitual de la ciudad</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>1-1-2021</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1209,12 +1205,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Banco de España, Síntesis de indicadores del mercado de la vivienda (SI_1_5)</t>
+          <t>Observatori Metropolità de l'Habitatge de Barcelona (O-HB)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>propio (elaboración del proyecto)</t>
         </is>
       </c>
       <c r="K12" s="3">
@@ -1223,7 +1219,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>script de origen: output/v17/f5/hechos.json:V17-B5-PRECIO-RENTA</t>
+          <t>script de origen: output/v17/f5/hechos.json:V17-DOC-OHB-GT-ALQUILER-BCN-2021</t>
         </is>
       </c>
       <c r="M12" s="4">
@@ -1295,31 +1291,31 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>V17-D3-AJUSTE-ESTADISTICO</t>
+          <t>V17-B5-LTV80</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Diferencia entre el residuo padronal y el saldo exterior oficial (revisiones, ruptura censal 2021, bajas por caducidad): -284.056 personas (2015-2024; INE ECP (ine_ecp_nacional.csv); INE MNP microdatos (data/raw/v11/ine_mnp); INE EVR/EMCR; dato de 2026-07-01; C4)</t>
+          <t>Préstamos con RPV mayor que 80 % (% del total), último dato: 9,6 % del total (2026-06; Banco de España, Síntesis de indicadores del mercado de la vivienda (SI_1_5); dato de 2026-06; C4)</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-284056</v>
+        <v>9.6</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>-84547</v>
+        <v>12.492</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>7161</v>
+        <v>17.025</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>personas</t>
+          <t>% del total</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2015-2024</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1329,12 +1325,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>INE ECP (ine_ecp_nacional.csv); INE MNP microdatos (data/raw/v11/ine_mnp); INE EVR/EMCR</t>
+          <t>Banco de España, Síntesis de indicadores del mercado de la vivienda (SI_1_5)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>INE</t>
+          <t>Banco de España</t>
         </is>
       </c>
       <c r="K14" s="3">
@@ -1343,7 +1339,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>script de origen: output/v17/f5/hechos.json:V17-D3-AJUSTE-ESTADISTICO</t>
+          <t>script de origen: output/v17/f5/hechos.json:V17-B5-LTV80</t>
         </is>
       </c>
       <c r="M14" s="4">

</xml_diff>